<commit_message>
WATSAN DI data: report village error noted (Malani = Gunogi, Nimbujhard = Chopriyal 2); Arakot 1 DI line disconnected
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -1826,7 +1826,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>broken</t>
+          <t>disconnected</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated. The report places Malani at Chopdiyal Gaon (field GPS: Gunogi), so its row may belong to Nimbujhard.</t>
+          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated. The report prints Chopdiyal Gaon as the village; Malani is at Gunogi (report error, confirmed by Rajat).</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated. The report places Nimbujhard at Gunogi (field GPS: Chopriyal), so its row may belong to Malani.</t>
+          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated. The report prints Gunogi as the village; Nimbujhard is at Chopriyal 2 (report error, confirmed by Rajat).</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>

</xml_diff>

<commit_message>
WATSAN DI data: Arakot 2 linked to Paniyar Dhar as well as Balench; shared handpump water counted once
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8 DI springs from the WATSAN Spring Assessment Report and the SRHU reports, plus Paniyar Dhar (no DI) as a comparison spring next to Balench. Kokhliyal is a Himmotthan site without DI, so it is not included.</t>
+          <t>9 DI springs from the WATSAN Spring Assessment Report and the SRHU reports. Arakot 2 may feed both Balench and Paniyar Dhar, so it is listed under both; count its water once. Kokhliyal is a Himmotthan site without DI, so it is not included.</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Comparison spring (no DI)</t>
+          <t>DI site</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1285,10 +1285,14 @@
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>FV26-DI-ARK2</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>No DI feeds it directly; Arakot 2 is nearest but not established (Rajat 2026-10-22)</t>
+          <t>Arakot 2 may feed Paniyar Dhar as well as Balench (Rajat, 2026-10-24); not verified</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1608,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y10"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2413,12 +2417,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FV26-DI-KAN</t>
+          <t>FV26-DI-ARK2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>WDI-07</t>
+          <t>WDI-06</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2428,33 +2432,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Kanatal</t>
+          <t>Arakot 2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>30.419538</t>
+          <t>30.365313</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>78.325791</t>
+          <t>78.379288</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2407.8</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>385</t>
-        </is>
+          <t>1796.6</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>99</v>
+      </c>
+      <c r="I8" t="n">
+        <v>258</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -2462,9 +2462,13 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>200</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
+        <v>150</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Form gives 300 m2 for Arakot 1 and 2 together; split evenly</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
           <t>Concrete</t>
@@ -2482,14 +2486,10 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>working</t>
+          <t>not_checked</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -2500,12 +2500,12 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>reported, not verified</t>
+          <t>reported, not verified; nearest DI to Paniyar Dhar but link to it not established</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -2515,19 +2515,19 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Working; Roadside, heavy litter; safety flag: clogging/dirty inflow; Depth on the form 100 m, reduced by 30 m (Rajat 2026-10-23: form depths were recorded about 30 m high)</t>
+          <t>Pump condition not recorded; Tested during visit; Depth on the form 100 m, reduced by 30 m (Rajat 2026-10-23: form depths were recorded about 30 m high)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FV26-DI-KUN</t>
+          <t>FV26-DI-KAN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WDI-08</t>
+          <t>WDI-07</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2537,51 +2537,65 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Kunjapuri</t>
+          <t>Kanatal</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>30.173165</t>
+          <t>30.419538</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>78.313007</t>
+          <t>78.325791</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1559.6</t>
+          <t>2407.8</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>152</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>189</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+          <t>385</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>200</v>
+      </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Concrete</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>not_checked</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr">
         <is>
           <t>working</t>
@@ -2595,12 +2609,12 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Reported by WATSAN/SRHU report; spring not seen on the visit (water tapped directly)</t>
+          <t>reported, not verified</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -2610,19 +2624,19 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Water tapped directly from the handpump; Working (recent DI on a previously defunct handpump); Exposed plastic roof pipes; animal and monkey damage risk</t>
+          <t>Working; Roadside, heavy litter; safety flag: clogging/dirty inflow; Depth on the form 100 m, reduced by 30 m (Rajat 2026-10-23: form depths were recorded about 30 m high)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SRC028-DI-DUN</t>
+          <t>FV26-DI-KUN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WDI-09</t>
+          <t>WDI-08</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2632,42 +2646,137 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Dungsi (Domsi)</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>30.481472</v>
-      </c>
-      <c r="F10" t="n">
-        <v>78.236694</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+          <t>Kunjapuri</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>30.173165</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>78.313007</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1559.6</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>not_checked</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>not_checked</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>working</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
       <c r="W10" t="inlineStr">
         <is>
+          <t>Reported by WATSAN/SRHU report; spring not seen on the visit (water tapped directly)</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Water tapped directly from the handpump; Working (recent DI on a previously defunct handpump); Exposed plastic roof pipes; animal and monkey damage risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SRC028-DI-DUN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WDI-09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dungsi (Domsi)</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>30.481472</v>
+      </c>
+      <c r="F11" t="n">
+        <v>78.236694</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
           <t>Reported by the SRHU Dungsi &amp; Makhdet report (SRC-028); not visited</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>SRHU Dungsi &amp; Makhdet hydrogeology report (SRC-028); handpump printed as 30°28'53.3"N 78°14'12.1"E</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2680,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6271,7 +6380,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>No DI. People said the flow has stayed similar: it dries every summer.</t>
+          <t>People said the flow has stayed similar: it still dries every summer.</t>
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
@@ -6341,7 +6450,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>No DI. People said the flow has stayed similar: it dries every summer.</t>
+          <t>People said the flow has stayed similar: it still dries every summer.</t>
         </is>
       </c>
       <c r="O54" t="inlineStr"/>
@@ -6360,12 +6469,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>village</t>
+          <t>handpump</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>WDI-06</t>
+          <t>FV26-DI-ARK2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6385,19 +6494,19 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>village_change</t>
+          <t>pump_status</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Still dries every summer</t>
+          <t>not_checked</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -6407,19 +6516,11 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Dries in lean months; people fetch water from Balench | No DI here: comparison spring.</t>
-        </is>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>access</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>same</t>
-        </is>
-      </c>
+          <t>Pump condition not recorded</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6429,17 +6530,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>WDI-07</t>
+          <t>WDI-06</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>handpump</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>RDI-SPR-0007</t>
+          <t>FV26-DI-ARK2</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6459,14 +6560,14 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="J56" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>~16</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -6481,7 +6582,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated.</t>
+          <t>Report's 'nearby DI handpump at higher elevation'; date and method not stated.</t>
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
@@ -6495,17 +6596,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>WDI-07</t>
+          <t>WDI-06</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>village</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>RDI-SPR-0007</t>
+          <t>WDI-06</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6520,28 +6621,24 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>flow_lpm</t>
-        </is>
-      </c>
-      <c r="I57" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="J57" t="n">
-        <v>21.72</v>
-      </c>
+          <t>village_change</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2 L in 5.8 s; 2 L in 5.5 s; 2 L in 5.3 s</t>
+          <t>Still dries every summer</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -6551,11 +6648,19 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Mean of 3 bucket-and-stopwatch readings, whole flow caught at the outlet pipe.</t>
-        </is>
-      </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
+          <t>Dries in lean months; people fetch water from Balench | Arakot 2 DI may feed this spring; no change reported.</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6580,7 +6685,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>field_visit_2026_10</t>
+          <t>watsan_report</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6588,40 +6693,36 @@
           <t>after_di</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>lean_flow_lpm</t>
+          <t>flow_lpm</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J58" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>10-15 L/min</t>
+          <t>~16</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>report</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
+          <t>WATSAN Spring Assessment Report (SRC-003), summary table; date and method not stated</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Typical flow people gave for this season now.</t>
+          <t>Report says DI was fitted at nearby handpumps; season of the reading is not stated.</t>
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
@@ -6665,23 +6766,23 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>monsoon_flow_lpm</t>
+          <t>flow_lpm</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>20</v>
+        <v>21.72</v>
       </c>
       <c r="J59" t="n">
-        <v>25</v>
+        <v>21.72</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>20-25 L/min</t>
+          <t>2 L in 5.8 s; 2 L in 5.5 s; 2 L in 5.3 s</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -6691,7 +6792,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Typical flow people gave for this season now.</t>
+          <t>Mean of 3 bucket-and-stopwatch readings, whole flow caught at the outlet pipe.</t>
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
@@ -6735,14 +6836,18 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>reported_change</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+          <t>lean_flow_lpm</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>10</v>
+      </c>
+      <c r="J60" t="n">
+        <v>15</v>
+      </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>increase</t>
+          <t>10-15 L/min</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -6757,7 +6862,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>Flow compared with 10-20 years ago: More. Nearby houses use this spring; flow has increased</t>
+          <t>Typical flow people gave for this season now.</t>
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
@@ -6776,35 +6881,43 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>handpump</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>FV26-DI-KAN</t>
+          <t>RDI-SPR-0007</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>before_di_recall</t>
+          <t>field_visit_2026_10</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>before_di</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
+          <t>after_di</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>pump_status</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+          <t>monsoon_flow_lpm</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>20</v>
+      </c>
+      <c r="J61" t="n">
+        <v>25</v>
+      </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>no_water_dry_season</t>
+          <t>20-25 L/min</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -6814,12 +6927,12 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Field form, DOCC/WATSAN field visit, October 2026 (recalled on 2026-10-19)</t>
+          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Handpump has water in the dry season now (implies it did not before)</t>
+          <t>Typical flow people gave for this season now.</t>
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
@@ -6838,12 +6951,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>handpump</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>FV26-DI-KAN</t>
+          <t>RDI-SPR-0007</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6863,19 +6976,19 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>pump_status</t>
+          <t>reported_change</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>working</t>
+          <t>increase</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -6883,7 +6996,11 @@
           <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Flow compared with 10-20 years ago: More. Nearby houses use this spring; flow has increased</t>
+        </is>
+      </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
     </row>
@@ -6910,44 +7027,40 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>watsan_report</t>
+          <t>before_di_recall</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>after_di</t>
+          <t>before_di</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>flow_lpm</t>
-        </is>
-      </c>
-      <c r="I63" t="n">
-        <v>16</v>
-      </c>
-      <c r="J63" t="n">
-        <v>16</v>
-      </c>
+          <t>pump_status</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>no_water_dry_season</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>report</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>WATSAN Spring Assessment Report (SRC-003), summary table; date and method not stated</t>
+          <t>Field form, DOCC/WATSAN field visit, October 2026 (recalled on 2026-10-19)</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Report's 'nearby DI handpump at higher elevation'; date and method not stated.</t>
+          <t>Handpump has water in the dry season now (implies it did not before)</t>
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
@@ -6991,19 +7104,19 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>village_change</t>
+          <t>pump_status</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Has water in the dry season; very good quality, travellers drink and wash</t>
+          <t>working</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -7011,21 +7124,9 @@
           <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>Handpump had no water in the dry season</t>
-        </is>
-      </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t>access</t>
-        </is>
-      </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>better</t>
-        </is>
-      </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7040,17 +7141,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>handpump</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>RDI-SPR-0007</t>
+          <t>FV26-DI-KAN</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>field_visit_2026_10</t>
+          <t>watsan_report</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7058,48 +7159,40 @@
           <t>after_di</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>village_change</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
+          <t>flow_lpm</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>16</v>
+      </c>
+      <c r="J65" t="n">
+        <v>16</v>
+      </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Flow has increased</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>report</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
+          <t>WATSAN Spring Assessment Report (SRC-003), summary table; date and method not stated</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Lower spring flow</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>access</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr">
-        <is>
-          <t>better</t>
-        </is>
-      </c>
+          <t>Report's 'nearby DI handpump at higher elevation'; date and method not stated.</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7109,7 +7202,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>WDI-08</t>
+          <t>WDI-07</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -7119,30 +7212,34 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>FV26-DI-KUN</t>
+          <t>FV26-DI-KAN</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>before_di_recall</t>
+          <t>field_visit_2026_10</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>before_di</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
+          <t>after_di</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>pump_status</t>
+          <t>village_change</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>defunct</t>
+          <t>Has water in the dry season; very good quality, travellers drink and wash</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -7152,16 +7249,24 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Field form, DOCC/WATSAN field visit, October 2026 (recalled on 2026-10-21)</t>
+          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>DI was fitted on a previously defunct handpump</t>
-        </is>
-      </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
+          <t>Handpump had no water in the dry season</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>better</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7171,17 +7276,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>WDI-08</t>
+          <t>WDI-07</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>handpump</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>FV26-DI-KUN</t>
+          <t>RDI-SPR-0007</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7196,24 +7301,24 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>pump_status</t>
+          <t>village_change</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>working</t>
+          <t>Flow has increased</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -7223,11 +7328,19 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Water tapped directly from the handpump</t>
-        </is>
-      </c>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
+          <t>Lower spring flow</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>better</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7252,52 +7365,180 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>field_visit_2026_10</t>
+          <t>before_di_recall</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>after_di</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>before_di</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>village_change</t>
+          <t>pump_status</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
+          <t>defunct</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Field form, DOCC/WATSAN field visit, October 2026 (recalled on 2026-10-21)</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>DI was fitted on a previously defunct handpump</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>OBS-068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>WDI-08</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>handpump</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>FV26-DI-KUN</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>field_visit_2026_10</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>after_di</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>pump_status</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>working</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Field form, DOCC/WATSAN field visit, October 2026</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Water tapped directly from the handpump</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>OBS-069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>WDI-08</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>handpump</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>FV26-DI-KUN</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>field_visit_2026_10</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>after_di</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>village_change</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
           <t>Handpump working; water tapped directly</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr">
+      <c r="L70" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="M70" t="inlineStr">
         <is>
           <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
+      <c r="N70" t="inlineStr">
         <is>
           <t>Handpump defunct</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr">
+      <c r="O70" t="inlineStr">
         <is>
           <t>access</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr">
+      <c r="P70" t="inlineStr">
         <is>
           <t>better</t>
         </is>

</xml_diff>

<commit_message>
DI Dashboard overview: equipment ribbon = handpumps working, DI lines connected, filters working, other work, each with a pop-up of sites needing work; drop latest spring records and work-to-follow-up panels (Rajat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -1846,7 +1846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1982,10 +1982,20 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
+          <t>other_work</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>di_note</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>location_class</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>location_note</t>
         </is>
@@ -2112,12 +2122,18 @@
           <t>Has water in the dry season; water decent, slight iron. Rooftop pipe broken, so the DI line is disconnected.</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Roof pipe broken</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
         <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2236,12 +2252,18 @@
           <t>DI tested on the visit. Linked to both Balench and Paniyar Dhar (not verified).</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Tested during visit</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2364,12 +2386,18 @@
           <t>DI line, gutter and filter in good order.</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2494,12 +2522,18 @@
           <t>Handpump broken (possible vehicle damage). First flush not working, filter blocked.</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Pump broken</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
         <is>
           <t>outside</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Geologist found no connection between this handpump and the naula.</t>
         </is>
@@ -2628,10 +2662,20 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
+          <t>Test the handpump water for iron</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2744,10 +2788,20 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
+          <t>Test the handpump water (quality improved, but no lab test yet)</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>house construction</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2862,12 +2916,18 @@
           <t>DI tested on the visit. Linked to both Balench and Paniyar Dhar (not verified).</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Tested during visit</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
         <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -2988,10 +3048,20 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
+          <t>Clean the roadside DI site (litter, dirty inflow)</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -3098,10 +3168,20 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
+          <t>Protect the exposed roof pipes from animals and monkeys</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Working (recent DI on a previously defunct handpump)</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
           <t>in_catchment</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
@@ -3176,6 +3256,8 @@
       </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
WATSAN DI data: rebuilt with IMD rain over all 25 years
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -761,11 +761,11 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>72.9</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1031,11 +1031,11 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1166,11 +1166,11 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>1446</v>
+        <v>1439</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1293,11 +1293,11 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N6" t="n">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1428,11 +1428,11 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N7" t="n">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>72.9</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1559,11 +1559,11 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N8" t="n">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1682,11 +1682,11 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>1446</v>
+        <v>1439</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N9" t="n">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1785,11 +1785,11 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025 (24 years; missing 2012)</t>
+          <t>IMD gridded rain gauges, mean of 2001-2025</t>
         </is>
       </c>
       <c r="N10" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">

</xml_diff>

<commit_message>
DI Dashboard: Spring column in the handpump table, Arakot 2 as one row with both springs; Track impact tabs ordered water injected, handpump, spring, DI and maintenance, impact beyond water (Rajat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -2249,7 +2249,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>DI tested on the visit. Linked to both Balench and Paniyar Dhar (not verified).</t>
+          <t>DI tested on the visit. Link to both springs not verified yet.</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr"/>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>DI tested on the visit. Linked to both Balench and Paniyar Dhar (not verified).</t>
+          <t>DI tested on the visit. Link to both springs not verified yet.</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr"/>

</xml_diff>

<commit_message>
WATSAN DI data: Makhdet/Dungsi left out (DI not installed yet); install years 2025 (Kunjapuri 2026), households and people (x5), Kaddukhal DI line intact, Chopriyal 2 first flush checked with orange-yellow water, Kunjapuri bore depth 60 m (Rajat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9 DI springs from the WATSAN Spring Assessment Report and the SRHU reports. Arakot 2 may feed both Balench and Paniyar Dhar, so it is listed under both; count its water once. Kokhliyal is a Himmotthan site without DI, so it is not included.</t>
+          <t>8 DI springs from the WATSAN Spring Assessment Report and the SRHU Badera report. Makhdet (Dungsi) is left out until its DI is installed. Arakot 2 may feed both Balench and Paniyar Dhar, so it is listed under both; count its water once. Kokhliyal is a Himmotthan site without DI, so it is not included.</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -786,8 +786,12 @@
           <t>19</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="R2" t="n">
+        <v>10</v>
+      </c>
+      <c r="S2" t="n">
+        <v>50</v>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
           <t>FV26-DI-ARK1;FV26-DI-ARK2</t>
@@ -917,15 +921,11 @@
           <t>39</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
+      <c r="R3" t="n">
+        <v>27</v>
+      </c>
+      <c r="S3" t="n">
+        <v>135</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Families once walked 2-3 km downhill for water. Today all 28 households (about 200 people) have water in the village, and it now supports vegetation and farming. People also report more water in springs further downhill at Silogi. The Himmotthan solar pumping scheme works alongside DI here.</t>
+          <t>Families once walked 2-3 km downhill for water. Today all 27 households (about 135 people) have water in the village, and it now supports vegetation and farming. People also report more water in springs further downhill at Silogi. The Himmotthan solar pumping scheme works alongside DI here.</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -1191,8 +1191,12 @@
           <t>29</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" t="n">
+        <v>75</v>
+      </c>
       <c r="T5" t="inlineStr">
         <is>
           <t>FV26-DI-GUN</t>
@@ -1323,7 +1327,9 @@
           <t>20</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>100</v>
+      </c>
       <c r="T6" t="inlineStr">
         <is>
           <t>FV26-DI-CHP2</t>
@@ -1453,8 +1459,12 @@
           <t>22</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="R7" t="n">
+        <v>5</v>
+      </c>
+      <c r="S7" t="n">
+        <v>25</v>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
           <t>FV26-DI-ARK2</t>
@@ -1584,8 +1594,12 @@
           <t>131</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+      <c r="R8" t="n">
+        <v>15</v>
+      </c>
+      <c r="S8" t="n">
+        <v>75</v>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
           <t>FV26-DI-KAN</t>
@@ -1707,8 +1721,12 @@
           <t>5</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="R9" t="n">
+        <v>15</v>
+      </c>
+      <c r="S9" t="n">
+        <v>75</v>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
           <t>FV26-DI-KUN</t>
@@ -1735,105 +1753,6 @@
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WDI-09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>RDI-SPR-0009</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>DI site</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Makhdet</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Makhdet (Dungsi &amp; Makhdet; also spelt Madkhet, Domsi)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Tehri Garhwal</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>30.482739</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>78.234675</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>1479.6</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>1330</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>IMD gridded rain gauges, mean of 2001-2025</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>2105</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>71.6</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>232.3</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>SRC028-DI-DUN</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Reported by the SRHU report (SRC-028); not visited</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>91.07</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1846,7 +1765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AD10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2065,8 +1984,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2203,8 +2128,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2329,8 +2260,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="N4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2468,7 +2405,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Installed last year for the school (field visit, 20 Oct 2026)</t>
+          <t>Installed last year for the school (field visit, 20 Oct 2026; Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2493,7 +2430,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>connected</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -2519,7 +2456,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Handpump broken (possible vehicle damage). First flush not working, filter blocked.</t>
+          <t>Handpump broken (possible vehicle damage). DI line intact; first flush not working, filter blocked.</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr"/>
@@ -2603,8 +2540,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2737,11 +2680,17 @@
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -2783,7 +2732,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Water quality improved: it was red/brown with high iron before DI (no lab test). DI line disconnected during house construction; filter blocked.</t>
+          <t>Water still orange-yellow at the first flush, but it was red before DI, so it is at least diluted now (no lab test). DI line disconnected during house construction; filter blocked.</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -2867,8 +2816,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2993,8 +2948,14 @@
           <t>Concrete</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
           <t>ok</t>
@@ -3113,12 +3074,20 @@
           <t>189</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>60</v>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
           <t>not_checked</t>
@@ -3186,78 +3155,6 @@
           <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SRC028-DI-DUN</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>WDI-09</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Dungsi (Domsi)</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>30.481472</v>
-      </c>
-      <c r="F11" t="n">
-        <v>78.236694</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>working</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Reported by the SRHU Dungsi &amp; Makhdet report (SRC-028); not visited</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>SRHU Dungsi &amp; Makhdet hydrogeology report (SRC-028); handpump printed as 30°28'53.3"N 78°14'12.1"E</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Not visited; Working (Rajat, 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>Not visited; from the SRHU report.</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3270,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5066,7 +4963,7 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Water available in the village for all 28 households (about 200 people)</t>
+          <t>Water available in the village for all 27 households (about 135 people)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -9318,126 +9215,6 @@
           <t>better</t>
         </is>
       </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>OBS-089</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>WDI-09</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>handpump</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>SRC028-DI-DUN</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>before_di_agreed</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>before_di</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>pump_status</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>defunct</t>
-        </is>
-      </c>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>agreed</t>
-        </is>
-      </c>
-      <c r="M90" t="inlineStr">
-        <is>
-          <t>All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>OBS-090</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>WDI-09</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>handpump</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>SRC028-DI-DUN</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>after_di_agreed</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>after_di</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>pump_status</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>working</t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>agreed</t>
-        </is>
-      </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t>All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>Not visited; Working (Rajat, 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="O91" t="inlineStr"/>
-      <c r="P91" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
WATSAN DI data: roof areas confirmed (Arakot 1 and 2 150 m2 each, Gunogi 120, Kunjapuri 150); Badeda flow recorded as not measured, spring covered (Rajat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -1976,7 +1976,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Form gives 300 m2 for Arakot 1 and 2 together; split evenly</t>
+          <t>150 m2 each for Arakot 1 and 2 (Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Form gives 300 m2 for Arakot 1 and 2 together; split evenly</t>
+          <t>150 m2 each for Arakot 1 and 2 (Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Form value unclear</t>
+          <t>Form value hard to read; 120 m2 kept (Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Form gives 300 m2 for Arakot 1 and 2 together; split evenly</t>
+          <t>150 m2 each for Arakot 1 and 2 (Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -3077,8 +3077,14 @@
       <c r="J10" t="n">
         <v>60</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>150</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
         <v>2026</v>
@@ -3167,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P89"/>
+  <dimension ref="A1:P90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9027,52 +9033,48 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>handpump</t>
+          <t>spring</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>FV26-DI-KUN</t>
+          <t>RDI-SPR-0008</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>before_di_agreed</t>
+          <t>rajat_2026_10_24</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>before_di</t>
+          <t>after_di</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>pump_status</t>
+          <t>flow_lpm</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr">
         <is>
-          <t>defunct</t>
+          <t>Not measured yet: the spring is covered, so there is no access to the outlet</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>agreed</t>
+          <t>not_measured</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>DI was fitted on a previously defunct handpump</t>
-        </is>
-      </c>
+          <t>Rajat, 2026-10-24</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr"/>
     </row>
@@ -9099,19 +9101,15 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>field_visit_2026_10</t>
+          <t>before_di_agreed</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>after_di</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>before_di</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>pump_status</t>
@@ -9121,7 +9119,7 @@
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
-          <t>working</t>
+          <t>defunct</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -9131,12 +9129,12 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Field form, DOCC/WATSAN field visit, October 2026; All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
+          <t>All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>Water tapped directly from the handpump</t>
+          <t>DI was fitted on a previously defunct handpump</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -9180,37 +9178,103 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>village_change</t>
+          <t>pump_status</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
+          <t>working</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>agreed</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Field form, DOCC/WATSAN field visit, October 2026; All WATSAN DI handpumps were defunct before DI (Rajat, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Water tapped directly from the handpump</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>OBS-089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>WDI-08</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>handpump</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>FV26-DI-KUN</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>field_visit_2026_10</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>after_di</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>village_change</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
           <t>Handpump working; water tapped directly</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr">
+      <c r="L90" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
+      <c r="M90" t="inlineStr">
         <is>
           <t>Field form, DOCC/WATSAN field visit, October 2026</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr">
+      <c r="N90" t="inlineStr">
         <is>
           <t>Handpump defunct</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr">
+      <c r="O90" t="inlineStr">
         <is>
           <t>access</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P90" t="inlineStr">
         <is>
           <t>better</t>
         </is>

</xml_diff>

<commit_message>
WATSAN DI data: Kunjapuri handpump renamed Badeda; its filter and first flush working and clean (most recent DI) (Rajat)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0132kAvxEJWuc4g7chmvtKAs
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -3046,7 +3046,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Kunjapuri</t>
+          <t>Badeda</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3096,12 +3096,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>Working again; people tap water directly. Exposed roof pipes at risk from animals and monkeys.</t>
+          <t>Most recent DI (2026); filter and first flush clean. Working again; people tap water directly. Exposed roof pipes at risk from animals and monkeys.</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard takes each DI handpump's location from the spring planner
The dashboard used "in the catchment" for every handpump, so Kanatal showed
about 29 m3/yr reaching Rasanulikhal while the planner showed about 114
(Kanatal sits in recharge zone R1). scripts/planner_di_locations.py runs the
planner once per WATSAN DI spring with its handpumps and stores each
handpump's location class; build_watsan_di_sites.py now reads it. Kaddukhal
stays "outside" (geologist found no link). Arakot 2 at Balench becomes
"outside", as in the planner.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYEMBaPiJtYrK4Gc2Fn2t3
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -2060,7 +2060,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>in_catchment</t>
+          <t>outside</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>Outside the spring's catchment and its recharge zones: the water will mostly feed other springs or streams. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>in_catchment</t>
+          <t>in_zone_slope</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>Inside recharge zone R1, on the slope that drains to the spring: most of the injected water can reach it. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard takes each DI handpump's location from the spring planner (#34)
The dashboard used "in the catchment" for every handpump, so Kanatal showed
about 29 m3/yr reaching Rasanulikhal while the planner showed about 114
(Kanatal sits in recharge zone R1). scripts/planner_di_locations.py runs the
planner once per WATSAN DI spring with its handpumps and stores each
handpump's location class; build_watsan_di_sites.py now reads it. Kaddukhal
stays "outside" (geologist found no link). Arakot 2 at Balench becomes
"outside", as in the planner.


Claude-Session: https://claude.ai/code/session_01SYEMBaPiJtYrK4Gc2Fn2t3

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
+++ b/data/02_processed/watsan_di/watsan_di_sites_v1.xlsx
@@ -2060,7 +2060,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>in_catchment</t>
+          <t>outside</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>Outside the spring's catchment and its recharge zones: the water will mostly feed other springs or streams. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -3019,12 +3019,12 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>in_catchment</t>
+          <t>in_zone_slope</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>Inside recharge zone R1, on the slope that drains to the spring: most of the injected water can reach it. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>Above the spring with a reported link; the planner's recharge zones are not run for this site yet, so the 'in the catchment' share is used.</t>
+          <t>In the surface catchment but outside the top recharge zones: little of the water is likely to reach this spring. (Spring planner, 2026-10-24.)</t>
         </is>
       </c>
     </row>

</xml_diff>